<commit_message>
Cleaned data in Excel docs including updating column names and changing data types. Also checked data for any inconsistencies
</commit_message>
<xml_diff>
--- a/Excel Files/Average_Days_Since_Claim_By_Product.xlsx
+++ b/Excel Files/Average_Days_Since_Claim_By_Product.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d9439836fb34a33/Documents/sales-analysis-project/Excel Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{598D02C5-8CD5-47AB-99AF-2A8B9F25C814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{598D02C5-8CD5-47AB-99AF-2A8B9F25C814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A00A0075-00BA-4CBC-9AC1-A6742170C448}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E65EE551-AAD0-4377-837C-CB1CC3972072}"/>
   </bookViews>
@@ -22,12 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
-    <t>Product_Name</t>
-  </si>
-  <si>
-    <t>average_days_sale_claim</t>
-  </si>
-  <si>
     <t>AirPods (2nd Generation)</t>
   </si>
   <si>
@@ -290,6 +284,12 @@
   </si>
   <si>
     <t>Smart Keyboard Folio</t>
+  </si>
+  <si>
+    <t>Name of Product</t>
+  </si>
+  <si>
+    <t>Average Number of Days between Sale and Claim</t>
   </si>
 </sst>
 </file>
@@ -773,8 +773,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -831,6 +833,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1153,718 +1159,719 @@
   <dimension ref="A1:B89"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="25" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.6328125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" s="1">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B3" s="1">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
-        <v>842</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B4" s="1">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
+      <c r="B5" s="1">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="1">
         <v>776</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="1">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="1">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="1">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="1">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="1">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="1">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="1">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="1">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="1">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="1">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="1">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="1">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="1">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="1">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="1">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="1">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="1">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="1">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="1">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="1">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="1">
         <v>832</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>812</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>768</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="1">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="1">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="1">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" s="1">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" s="1">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" s="1">
         <v>789</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>785</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>776</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>808</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12">
-        <v>825</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" s="1">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B39" s="1">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" s="1">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" s="1">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="1">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" s="1">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" s="1">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" s="1">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47" s="1">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B48" s="1">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B49" s="1">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" s="1">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B51" s="1">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B52" s="1">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B53" s="1">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B54" s="1">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B55" s="1">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B56" s="1">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B57" s="1">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B58" s="1">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B59" s="1">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B60" s="1">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61" s="1">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B62" s="1">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B63" s="1">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B64" s="1">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B65" s="1">
         <v>781</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14">
-        <v>765</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15">
-        <v>782</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17">
-        <v>798</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18">
-        <v>830</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20">
-        <v>848</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21">
-        <v>807</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22">
-        <v>901</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>26</v>
-      </c>
-      <c r="B26">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27">
-        <v>838</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>28</v>
-      </c>
-      <c r="B28">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B66" s="1">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B67" s="1">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B68" s="1">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B69" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B70" s="1">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B71" s="1">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A72" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B72" s="1">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A73" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B73" s="1">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A74" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B74" s="1">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B75" s="1">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A76" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B76" s="1">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A77" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B77" s="1">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A78" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B78" s="1">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A79" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B79" s="1">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A80" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B80" s="1">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A81" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B81" s="1">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A82" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B82" s="1">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A83" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B83" s="1">
         <v>788</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29">
-        <v>828</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30">
-        <v>796</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31">
-        <v>832</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>32</v>
-      </c>
-      <c r="B32">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>33</v>
-      </c>
-      <c r="B33">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>34</v>
-      </c>
-      <c r="B34">
-        <v>809</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35">
-        <v>834</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>36</v>
-      </c>
-      <c r="B36">
-        <v>839</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>37</v>
-      </c>
-      <c r="B37">
-        <v>789</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>38</v>
-      </c>
-      <c r="B38">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>39</v>
-      </c>
-      <c r="B39">
-        <v>856</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>40</v>
-      </c>
-      <c r="B40">
-        <v>793</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>41</v>
-      </c>
-      <c r="B41">
-        <v>836</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>42</v>
-      </c>
-      <c r="B42">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>43</v>
-      </c>
-      <c r="B43">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>44</v>
-      </c>
-      <c r="B44">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45">
-        <v>844</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>46</v>
-      </c>
-      <c r="B46">
-        <v>797</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>47</v>
-      </c>
-      <c r="B47">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>49</v>
-      </c>
-      <c r="B49">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A84" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B84" s="1">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A85" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B85" s="1">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A86" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B86" s="1">
         <v>791</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>50</v>
-      </c>
-      <c r="B50">
-        <v>801</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>51</v>
-      </c>
-      <c r="B51">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>52</v>
-      </c>
-      <c r="B52">
-        <v>874</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>53</v>
-      </c>
-      <c r="B53">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>54</v>
-      </c>
-      <c r="B54">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>55</v>
-      </c>
-      <c r="B55">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>56</v>
-      </c>
-      <c r="B56">
-        <v>795</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>57</v>
-      </c>
-      <c r="B57">
-        <v>840</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>58</v>
-      </c>
-      <c r="B58">
-        <v>793</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>59</v>
-      </c>
-      <c r="B59">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>60</v>
-      </c>
-      <c r="B60">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>61</v>
-      </c>
-      <c r="B61">
-        <v>839</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>62</v>
-      </c>
-      <c r="B62">
-        <v>849</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>63</v>
-      </c>
-      <c r="B63">
-        <v>783</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>64</v>
-      </c>
-      <c r="B64">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
-        <v>65</v>
-      </c>
-      <c r="B65">
-        <v>781</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>66</v>
-      </c>
-      <c r="B66">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>67</v>
-      </c>
-      <c r="B67">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
-        <v>68</v>
-      </c>
-      <c r="B68">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>69</v>
-      </c>
-      <c r="B69">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>70</v>
-      </c>
-      <c r="B70">
-        <v>815</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
-        <v>71</v>
-      </c>
-      <c r="B71">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
-        <v>72</v>
-      </c>
-      <c r="B72">
-        <v>783</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>73</v>
-      </c>
-      <c r="B73">
-        <v>818</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>74</v>
-      </c>
-      <c r="B74">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>75</v>
-      </c>
-      <c r="B75">
-        <v>789</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>76</v>
-      </c>
-      <c r="B76">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>77</v>
-      </c>
-      <c r="B77">
-        <v>858</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
-        <v>78</v>
-      </c>
-      <c r="B78">
-        <v>833</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
-        <v>79</v>
-      </c>
-      <c r="B79">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>80</v>
-      </c>
-      <c r="B80">
-        <v>793</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
-        <v>81</v>
-      </c>
-      <c r="B81">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
-        <v>82</v>
-      </c>
-      <c r="B82">
-        <v>748</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
-        <v>83</v>
-      </c>
-      <c r="B83">
-        <v>788</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
-        <v>84</v>
-      </c>
-      <c r="B84">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A87" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B85">
-        <v>852</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+      <c r="B87" s="1">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A88" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B86">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+      <c r="B88" s="1">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A89" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B87">
-        <v>897</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
-        <v>88</v>
-      </c>
-      <c r="B88">
-        <v>779</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
-        <v>89</v>
-      </c>
-      <c r="B89">
+      <c r="B89" s="1">
         <v>783</v>
       </c>
     </row>

</xml_diff>